<commit_message>
fix: update Bug reporting.xlsx
</commit_message>
<xml_diff>
--- a/Bug reporting.xlsx
+++ b/Bug reporting.xlsx
@@ -5,22 +5,38 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\BismarkKadogbe\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\BismarkKadogbe\Desktop\Personal Projects\test project\Demoblaze\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{568708F3-998A-46D1-9770-F66E73519F7A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1D44144D-CE69-43DD-BD91-38A6A65B839D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="31410" yWindow="2145" windowWidth="17280" windowHeight="8880" xr2:uid="{190E49B9-9A5C-4FDD-9A68-FAE6B7B9C17C}"/>
+    <workbookView xWindow="14685" yWindow="-16320" windowWidth="29040" windowHeight="15720" xr2:uid="{190E49B9-9A5C-4FDD-9A68-FAE6B7B9C17C}"/>
   </bookViews>
   <sheets>
-    <sheet name="Bug reporting" sheetId="1" r:id="rId1"/>
+    <sheet name="Dashboard" sheetId="3" r:id="rId1"/>
+    <sheet name="Smoke Suite" sheetId="4" r:id="rId2"/>
+    <sheet name="Regression Suite" sheetId="5" r:id="rId3"/>
+    <sheet name="Bug Log" sheetId="6" r:id="rId4"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="54">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="190" uniqueCount="145">
   <si>
     <t>Defect ID</t>
   </si>
@@ -64,12 +80,6 @@
     <t>Assigned To</t>
   </si>
   <si>
-    <t>Date Closed</t>
-  </si>
-  <si>
-    <t>Resolution</t>
-  </si>
-  <si>
     <t>BUG-001</t>
   </si>
   <si>
@@ -91,9 +101,6 @@
     <t>Open</t>
   </si>
   <si>
-    <t>1. Open Sign Up modal 2. Enter existing username 3. Click Sign Up</t>
-  </si>
-  <si>
     <t>Alert should read "This user already exists."</t>
   </si>
   <si>
@@ -103,9 +110,6 @@
     <t>QA Team</t>
   </si>
   <si>
-    <t>Dev Team</t>
-  </si>
-  <si>
     <t>—</t>
   </si>
   <si>
@@ -121,15 +125,9 @@
     <t>Cart total displays without currency symbol</t>
   </si>
   <si>
-    <t>Cart row shows "820" instead of "\$820" while product page shows "\$820"</t>
-  </si>
-  <si>
     <t>Chrome 124</t>
   </si>
   <si>
-    <t>1. Add product to cart 2. Navigate to cart</t>
-  </si>
-  <si>
     <t>Price format should be consistent</t>
   </si>
   <si>
@@ -151,9 +149,6 @@
     <t>P2</t>
   </si>
   <si>
-    <t>1. Add item to cart 2. Go to cart 3. Click Delete</t>
-  </si>
-  <si>
     <t>Immediate removal without full reload</t>
   </si>
   <si>
@@ -175,20 +170,391 @@
     <t>Guest able to make purchase</t>
   </si>
   <si>
-    <t>1. Complete checkout 2.Click purchase 3. Observe confirmation dialog</t>
-  </si>
-  <si>
     <t>It should redirect the user to login</t>
   </si>
   <si>
-    <t>Purchase shows success even for guest users</t>
+    <t>Total Test Cases</t>
+  </si>
+  <si>
+    <t>&lt; 30 min</t>
+  </si>
+  <si>
+    <t>Comprehensive validation of all functional areas.</t>
+  </si>
+  <si>
+    <t>Regression Test Suite (@regression)</t>
+  </si>
+  <si>
+    <t>&lt; 5 min</t>
+  </si>
+  <si>
+    <t>Provide rapid feedback on build stability.</t>
+  </si>
+  <si>
+    <t>Smoke Test Suite (@smoke)</t>
+  </si>
+  <si>
+    <t>Test Case Count</t>
+  </si>
+  <si>
+    <t>Target Duration</t>
+  </si>
+  <si>
+    <t>Objective</t>
+  </si>
+  <si>
+    <t>Test Suite / Tag</t>
+  </si>
+  <si>
+    <t>Total Test Cases:</t>
+  </si>
+  <si>
+    <t>Total Test Suites:</t>
+  </si>
+  <si>
+    <t>Demoblaze Product Store (https://www.demoblaze.com)</t>
+  </si>
+  <si>
+    <t>Application Under Test:</t>
+  </si>
+  <si>
+    <t>Demoblaze QA Test Suite Dashboard</t>
+  </si>
+  <si>
+    <t>- Product grid updates for each category
+- Correct category items are displayed</t>
+  </si>
+  <si>
+    <t>1. Click "Phones" category link
+2. Verify products filter to phones only
+3. Click "Laptops" category link
+4. Verify products filter to laptops only</t>
+  </si>
+  <si>
+    <t>Homepage is loaded</t>
+  </si>
+  <si>
+    <t>High</t>
+  </si>
+  <si>
+    <t>Validate Product Category Navigation</t>
+  </si>
+  <si>
+    <t>TC-SMOKE-005</t>
+  </si>
+  <si>
+    <t>- "Welcome" message disappears
+- "Log in" and "Sign up" buttons become visible
+- User session is terminated</t>
+  </si>
+  <si>
+    <t>1. Log in with valid credentials
+2. Click "Log out" in navbar</t>
+  </si>
+  <si>
+    <t>User is logged in</t>
+  </si>
+  <si>
+    <t>Verify Logout Functionality</t>
+  </si>
+  <si>
+    <t>TC-SMOKE-004</t>
+  </si>
+  <si>
+    <t>- Product appears in cart table
+- Product title matches selected item
+- Cart total is calculated correctly</t>
+  </si>
+  <si>
+    <t>1. Click on first product in the grid
+2. Verify product details page loads
+3. Click "Add to cart" button
+4. Accept browser alert confirmation
+5. Navigate to Cart page</t>
+  </si>
+  <si>
+    <t>User is on homepage, products are loaded</t>
+  </si>
+  <si>
+    <t>Critical</t>
+  </si>
+  <si>
+    <t>Confirm Product Can Be Added to Cart</t>
+  </si>
+  <si>
+    <t>- Login modal closes
+- "Welcome {username}" displayed in navbar
+- "Log out" option becomes visible</t>
+  </si>
+  <si>
+    <t>1. Navigate to homepage
+2. Click "Log in" button in navbar
+3. Enter valid username
+4. Enter valid password
+5. Click "Log in" submit button</t>
+  </si>
+  <si>
+    <t>Test user account exists</t>
+  </si>
+  <si>
+    <t>Validate User Login with Valid Credentials</t>
+  </si>
+  <si>
+    <t>TC-SMOKE-002</t>
+  </si>
+  <si>
+    <t>- Page title equals "STORE"
+- Navbar brand "PRODUCT STORE" is visible
+- Product grid contains at least 1 item
+- Footer is visible</t>
+  </si>
+  <si>
+    <t>1. Navigate to https://www.demoblaze.com/index.html
+2. Wait for page to fully load</t>
+  </si>
+  <si>
+    <t>Application is accessible</t>
+  </si>
+  <si>
+    <t>Verify Application Homepage Loads</t>
+  </si>
+  <si>
+    <t>TC-SMOKE-001</t>
+  </si>
+  <si>
+    <t>Expected Results</t>
+  </si>
+  <si>
+    <t>Test Steps</t>
+  </si>
+  <si>
+    <t>Preconditions</t>
+  </si>
+  <si>
+    <t>Test Case Title</t>
+  </si>
+  <si>
+    <t>Test Case ID</t>
+  </si>
+  <si>
+    <t>5.1 SMOKE TEST SUITE (@smoke)</t>
+  </si>
+  <si>
+    <t>- Confirmation dialog appears with order details
+- Order ID is generated and displayed
+- Amount matches cart total
+- "OK" button closes dialog and clears cart</t>
+  </si>
+  <si>
+    <t>1. Log in with valid credentials
+2. Add product to cart
+3. Navigate to Cart page
+4. Click "Place Order" button
+5. Fill in Name field
+6. Fill in Country field
+7. Fill in City field
+8. Fill in Credit Card field
+9. Fill in Month field
+10. Fill in Year field
+11. Click "Purchase" button</t>
+  </si>
+  <si>
+    <t>User is logged in, cart has items</t>
+  </si>
+  <si>
+    <t>Test Complete Checkout Process</t>
+  </si>
+  <si>
+    <t>- Product is removed from cart table
+- Cart total updates to $0 (if last item)
+- "Delete" link is no longer present</t>
+  </si>
+  <si>
+    <t>1. Add a product to cart
+2. Navigate to Cart page
+3. Click "Delete" link for the product
+4. Wait for page to refresh</t>
+  </si>
+  <si>
+    <t>Cart contains at least 1 product</t>
+  </si>
+  <si>
+    <t>Test Removing Product from Cart</t>
+  </si>
+  <si>
+    <t>- Both products appear in cart
+- Quantities are correct (1 each)
+- Total price equals sum of individual prices</t>
+  </si>
+  <si>
+    <t>1. Add Product A to cart
+2. Navigate back to homepage
+3. Add Product B to cart
+4. Navigate to Cart page</t>
+  </si>
+  <si>
+    <t>User is on homepage</t>
+  </si>
+  <si>
+    <t>Test Adding Multiple Products to Cart</t>
+  </si>
+  <si>
+    <t>TC-REG-007</t>
+  </si>
+  <si>
+    <t>- Only monitor products are displayed
+- Product count is greater than 0</t>
+  </si>
+  <si>
+    <t>1. Click "Monitors" in category menu
+2. Count number of products displayed</t>
+  </si>
+  <si>
+    <t>Homepage loaded with product catalog</t>
+  </si>
+  <si>
+    <t>Verify Product Search by Category - Monitors</t>
+  </si>
+  <si>
+    <t>TC-REG-006</t>
+  </si>
+  <si>
+    <t>- Only laptop products are displayed
+- Product count is greater than 0</t>
+  </si>
+  <si>
+    <t>1. Click "Laptops" in category menu
+2. Count number of products displayed
+3. Verify all displayed items are laptops</t>
+  </si>
+  <si>
+    <t>Verify Product Search by Category - Laptops</t>
+  </si>
+  <si>
+    <t>TC-REG-005</t>
+  </si>
+  <si>
+    <t>- Only phone products are displayed
+- Product count is greater than 0
+- No laptops or monitors appear</t>
+  </si>
+  <si>
+    <t>1. Click "Phones" in category menu
+2. Count number of products displayed
+3. Verify all displayed items are phones</t>
+  </si>
+  <si>
+    <t>Verify Product Search by Category - Phones</t>
+  </si>
+  <si>
+    <t>TC-REG-004</t>
+  </si>
+  <si>
+    <t>- Alert dialog displays "Please fill out Username and Password."
+- Registration is not processed</t>
+  </si>
+  <si>
+    <t>1. Navigate to homepage
+2. Click "Sign up" button
+3. Leave username empty
+4. Leave password empty
+5. Click "Sign up" submit button</t>
+  </si>
+  <si>
+    <t>None</t>
+  </si>
+  <si>
+    <t>Medium</t>
+  </si>
+  <si>
+    <t>Validate Registration with Empty Fields</t>
+  </si>
+  <si>
+    <t>TC-REG-003</t>
+  </si>
+  <si>
+    <t>- Alert dialog displays "This user already exist."
+- Account is not duplicated</t>
+  </si>
+  <si>
+    <t>1. Navigate to homepage
+2. Click "Sign up" button
+3. Enter existing username
+4. Enter valid password
+5. Click "Sign up" submit button</t>
+  </si>
+  <si>
+    <t>Username already exists in system</t>
+  </si>
+  <si>
+    <t>Validate Registration with Existing Username</t>
+  </si>
+  <si>
+    <t>- Alert dialog displays "Sign up successful."
+- New account can be used for login</t>
+  </si>
+  <si>
+    <t>1. Navigate to homepage
+2. Click "Sign up" button
+3. Enter unique username (timestamp-based)
+4. Enter valid password (8+ chars, alphanumeric)
+5. Click "Sign up" submit button</t>
+  </si>
+  <si>
+    <t>Username does not already exist</t>
+  </si>
+  <si>
+    <t>Validate User Registration with Valid Data</t>
+  </si>
+  <si>
+    <t>TC-REG-001</t>
+  </si>
+  <si>
+    <t>5.2 REGRESSION TEST SUITE (@regression)</t>
+  </si>
+  <si>
+    <t>DEFECT LOG / TRACKER</t>
+  </si>
+  <si>
+    <t>Date Close</t>
+  </si>
+  <si>
+    <t>DevTeam</t>
+  </si>
+  <si>
+    <t>07/05/2026</t>
+  </si>
+  <si>
+    <t>Purchase shows success even for guest user</t>
+  </si>
+  <si>
+    <t>1. Complete checkout
+2. Click purchase
+3. Observe confirmation dialog</t>
+  </si>
+  <si>
+    <t>1. Add item to cart
+2. Go to cart
+3. Click Delete</t>
+  </si>
+  <si>
+    <t>1. Add product to cart
+2. Navigate to cart</t>
+  </si>
+  <si>
+    <t>Cart row shows "820" instead of "$820" while product page shows "$820"</t>
+  </si>
+  <si>
+    <t>1. Open Sign Up modal
+2. Enter existing username
+3. Click Sign Up</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="19" x14ac:knownFonts="1">
+  <fonts count="27" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -324,13 +690,60 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="8"/>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <scheme val="minor"/>
+      <b/>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Segoe UI"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Segoe UI"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Segoe UI"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="16"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Segoe UI"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color rgb="FF833C0C"/>
+      <name val="Segoe UI"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color rgb="FFC65911"/>
+      <name val="Segoe UI"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="10"/>
+      <color rgb="FF595959"/>
+      <name val="Segoe UI"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="14"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Segoe UI"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color rgb="FF375623"/>
+      <name val="Segoe UI"/>
     </font>
   </fonts>
-  <fills count="33">
+  <fills count="41">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -510,8 +923,56 @@
         <bgColor indexed="65"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2F2F2"/>
+        <bgColor rgb="FFF2F2F2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF2F5597"/>
+        <bgColor rgb="FF2F5597"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF1F497D"/>
+        <bgColor rgb="FF1F497D"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFFF"/>
+        <bgColor rgb="FFFFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFF2CC"/>
+        <bgColor rgb="FFFFF2CC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF9FAFB"/>
+        <bgColor rgb="FFF9FAFB"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFCE4D6"/>
+        <bgColor rgb="FFFCE4D6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFE2EFDA"/>
+        <bgColor rgb="FFE2EFDA"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="10">
+  <borders count="11">
     <border>
       <left/>
       <right/>
@@ -626,6 +1087,21 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFD9D9D9"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFD9D9D9"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFD9D9D9"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFD9D9D9"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -671,9 +1147,66 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="18" fillId="33" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="33" borderId="10" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="18" fillId="33" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="34" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="18" fillId="33" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="21" fillId="35" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="36" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="36" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="37" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="38" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="38" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="39" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="33" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="35" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="40" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="38" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="36" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1048,275 +1581,813 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{18FCCFE8-0A68-4974-B86E-A7AEAE799DDB}">
-  <dimension ref="A1:P5"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D37814B6-018B-4C3E-BEB1-7EE274F5D4C7}">
+  <dimension ref="A1:D11"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="12.44140625" customWidth="1"/>
-    <col min="2" max="2" width="15.109375" customWidth="1"/>
-    <col min="3" max="3" width="51.21875" customWidth="1"/>
-    <col min="4" max="4" width="75.109375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="19.88671875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="57.88671875" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="38.77734375" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="34.6640625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8.5546875" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="11.21875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="38" customWidth="1"/>
+    <col min="2" max="2" width="50" customWidth="1"/>
+    <col min="3" max="4" width="18" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A1" t="s">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A1" s="11" t="s">
+        <v>60</v>
+      </c>
+      <c r="B1" s="10"/>
+      <c r="C1" s="10"/>
+      <c r="D1" s="10"/>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A2" s="10"/>
+      <c r="B2" s="10"/>
+      <c r="C2" s="10"/>
+      <c r="D2" s="10"/>
+    </row>
+    <row r="4" spans="1:4" ht="15" x14ac:dyDescent="0.35">
+      <c r="A4" s="9" t="s">
+        <v>59</v>
+      </c>
+      <c r="B4" s="8" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" ht="15" x14ac:dyDescent="0.35">
+      <c r="A5" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="B5" s="8">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" ht="15" x14ac:dyDescent="0.35">
+      <c r="A6" s="9" t="s">
+        <v>56</v>
+      </c>
+      <c r="B6" s="8">
+        <f>COUNTA('Smoke Suite'!A4:A8)+COUNTA('Regression Suite'!A4:A12)</f>
+        <v>14</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="A8" s="7" t="s">
+        <v>55</v>
+      </c>
+      <c r="B8" s="7" t="s">
+        <v>54</v>
+      </c>
+      <c r="C8" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="D8" s="7" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" ht="15" x14ac:dyDescent="0.3">
+      <c r="A9" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="B9" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="C9" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="D9" s="4">
+        <f>COUNTA('Smoke Suite'!A4:A8)</f>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" ht="15" x14ac:dyDescent="0.3">
+      <c r="A10" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="B10" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="C10" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="D10" s="4">
+        <f>COUNTA('Regression Suite'!A4:A12)</f>
+        <v>9</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" ht="15" x14ac:dyDescent="0.3">
+      <c r="A11" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="B11" s="2"/>
+      <c r="C11" s="2"/>
+      <c r="D11" s="1">
+        <f>SUM(D9:D10)</f>
+        <v>14</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:D2"/>
+    <mergeCell ref="A11:C11"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{89F87383-340E-4355-8FE8-4EC53C0E21F5}">
+  <dimension ref="A1:F8"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="16" customWidth="1"/>
+    <col min="2" max="2" width="45" customWidth="1"/>
+    <col min="3" max="3" width="44" customWidth="1"/>
+    <col min="4" max="5" width="45" customWidth="1"/>
+    <col min="6" max="6" width="12" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="19" t="s">
+        <v>92</v>
+      </c>
+      <c r="B1" s="10"/>
+      <c r="C1" s="10"/>
+      <c r="D1" s="10"/>
+      <c r="E1" s="10"/>
+    </row>
+    <row r="2" spans="1:6" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="18"/>
+      <c r="B2" s="10"/>
+      <c r="C2" s="10"/>
+      <c r="D2" s="10"/>
+      <c r="E2" s="10"/>
+    </row>
+    <row r="3" spans="1:6" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="7" t="s">
+        <v>91</v>
+      </c>
+      <c r="B3" s="7" t="s">
+        <v>90</v>
+      </c>
+      <c r="C3" s="7" t="s">
+        <v>89</v>
+      </c>
+      <c r="D3" s="7" t="s">
+        <v>88</v>
+      </c>
+      <c r="E3" s="7" t="s">
+        <v>87</v>
+      </c>
+      <c r="F3" s="7" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" ht="60" x14ac:dyDescent="0.3">
+      <c r="A4" s="12" t="s">
+        <v>86</v>
+      </c>
+      <c r="B4" s="13" t="s">
+        <v>85</v>
+      </c>
+      <c r="C4" s="13" t="s">
+        <v>84</v>
+      </c>
+      <c r="D4" s="13" t="s">
+        <v>83</v>
+      </c>
+      <c r="E4" s="13" t="s">
+        <v>82</v>
+      </c>
+      <c r="F4" s="17" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" ht="75" x14ac:dyDescent="0.3">
+      <c r="A5" s="15" t="s">
+        <v>81</v>
+      </c>
+      <c r="B5" s="16" t="s">
+        <v>80</v>
+      </c>
+      <c r="C5" s="16" t="s">
+        <v>79</v>
+      </c>
+      <c r="D5" s="16" t="s">
+        <v>78</v>
+      </c>
+      <c r="E5" s="16" t="s">
+        <v>77</v>
+      </c>
+      <c r="F5" s="17" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" ht="75" x14ac:dyDescent="0.3">
+      <c r="A6" s="12" t="s">
+        <v>27</v>
+      </c>
+      <c r="B6" s="13" t="s">
+        <v>76</v>
+      </c>
+      <c r="C6" s="13" t="s">
+        <v>74</v>
+      </c>
+      <c r="D6" s="13" t="s">
+        <v>73</v>
+      </c>
+      <c r="E6" s="13" t="s">
+        <v>72</v>
+      </c>
+      <c r="F6" s="17" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" ht="45" x14ac:dyDescent="0.3">
+      <c r="A7" s="15" t="s">
+        <v>71</v>
+      </c>
+      <c r="B7" s="16" t="s">
+        <v>70</v>
+      </c>
+      <c r="C7" s="16" t="s">
+        <v>69</v>
+      </c>
+      <c r="D7" s="16" t="s">
+        <v>68</v>
+      </c>
+      <c r="E7" s="16" t="s">
+        <v>67</v>
+      </c>
+      <c r="F7" s="14" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" ht="60" x14ac:dyDescent="0.3">
+      <c r="A8" s="12" t="s">
+        <v>66</v>
+      </c>
+      <c r="B8" s="13" t="s">
+        <v>65</v>
+      </c>
+      <c r="C8" s="13" t="s">
+        <v>63</v>
+      </c>
+      <c r="D8" s="13" t="s">
+        <v>62</v>
+      </c>
+      <c r="E8" s="13" t="s">
+        <v>61</v>
+      </c>
+      <c r="F8" s="14" t="s">
+        <v>64</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A2:E2"/>
+    <mergeCell ref="A1:E1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{98F033AE-F5E5-49BF-88B6-733276573AA1}">
+  <dimension ref="A1:F12"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="16" customWidth="1"/>
+    <col min="2" max="2" width="45" customWidth="1"/>
+    <col min="3" max="3" width="40" customWidth="1"/>
+    <col min="4" max="5" width="45" customWidth="1"/>
+    <col min="6" max="6" width="12" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="19" t="s">
+        <v>134</v>
+      </c>
+      <c r="B1" s="10"/>
+      <c r="C1" s="10"/>
+      <c r="D1" s="10"/>
+      <c r="E1" s="10"/>
+    </row>
+    <row r="2" spans="1:6" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="18"/>
+      <c r="B2" s="10"/>
+      <c r="C2" s="10"/>
+      <c r="D2" s="10"/>
+      <c r="E2" s="10"/>
+    </row>
+    <row r="3" spans="1:6" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="7" t="s">
+        <v>91</v>
+      </c>
+      <c r="B3" s="7" t="s">
+        <v>90</v>
+      </c>
+      <c r="C3" s="7" t="s">
+        <v>89</v>
+      </c>
+      <c r="D3" s="7" t="s">
+        <v>88</v>
+      </c>
+      <c r="E3" s="7" t="s">
+        <v>87</v>
+      </c>
+      <c r="F3" s="7" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" ht="75" x14ac:dyDescent="0.3">
+      <c r="A4" s="12" t="s">
+        <v>133</v>
+      </c>
+      <c r="B4" s="13" t="s">
+        <v>132</v>
+      </c>
+      <c r="C4" s="13" t="s">
+        <v>131</v>
+      </c>
+      <c r="D4" s="13" t="s">
+        <v>130</v>
+      </c>
+      <c r="E4" s="13" t="s">
+        <v>129</v>
+      </c>
+      <c r="F4" s="14" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" ht="75" x14ac:dyDescent="0.3">
+      <c r="A5" s="15" t="s">
+        <v>15</v>
+      </c>
+      <c r="B5" s="16" t="s">
+        <v>128</v>
+      </c>
+      <c r="C5" s="16" t="s">
+        <v>127</v>
+      </c>
+      <c r="D5" s="16" t="s">
+        <v>126</v>
+      </c>
+      <c r="E5" s="16" t="s">
+        <v>125</v>
+      </c>
+      <c r="F5" s="20" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" ht="75" x14ac:dyDescent="0.3">
+      <c r="A6" s="12" t="s">
+        <v>124</v>
+      </c>
+      <c r="B6" s="13" t="s">
+        <v>123</v>
+      </c>
+      <c r="C6" s="13" t="s">
+        <v>121</v>
+      </c>
+      <c r="D6" s="13" t="s">
+        <v>120</v>
+      </c>
+      <c r="E6" s="13" t="s">
+        <v>119</v>
+      </c>
+      <c r="F6" s="20" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" ht="45" x14ac:dyDescent="0.3">
+      <c r="A7" s="15" t="s">
+        <v>118</v>
+      </c>
+      <c r="B7" s="16" t="s">
+        <v>117</v>
+      </c>
+      <c r="C7" s="16" t="s">
+        <v>108</v>
+      </c>
+      <c r="D7" s="16" t="s">
+        <v>116</v>
+      </c>
+      <c r="E7" s="16" t="s">
+        <v>115</v>
+      </c>
+      <c r="F7" s="14" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" ht="45" x14ac:dyDescent="0.3">
+      <c r="A8" s="12" t="s">
+        <v>114</v>
+      </c>
+      <c r="B8" s="13" t="s">
+        <v>113</v>
+      </c>
+      <c r="C8" s="13" t="s">
+        <v>108</v>
+      </c>
+      <c r="D8" s="13" t="s">
+        <v>112</v>
+      </c>
+      <c r="E8" s="13" t="s">
+        <v>111</v>
+      </c>
+      <c r="F8" s="14" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" ht="30" x14ac:dyDescent="0.3">
+      <c r="A9" s="15" t="s">
+        <v>110</v>
+      </c>
+      <c r="B9" s="16" t="s">
+        <v>109</v>
+      </c>
+      <c r="C9" s="16" t="s">
+        <v>108</v>
+      </c>
+      <c r="D9" s="16" t="s">
+        <v>107</v>
+      </c>
+      <c r="E9" s="16" t="s">
+        <v>106</v>
+      </c>
+      <c r="F9" s="14" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" ht="60" x14ac:dyDescent="0.3">
+      <c r="A10" s="12" t="s">
+        <v>105</v>
+      </c>
+      <c r="B10" s="13" t="s">
+        <v>104</v>
+      </c>
+      <c r="C10" s="13" t="s">
+        <v>103</v>
+      </c>
+      <c r="D10" s="13" t="s">
+        <v>102</v>
+      </c>
+      <c r="E10" s="13" t="s">
+        <v>101</v>
+      </c>
+      <c r="F10" s="14" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" ht="60" x14ac:dyDescent="0.3">
+      <c r="A11" s="15" t="s">
+        <v>33</v>
+      </c>
+      <c r="B11" s="16" t="s">
+        <v>100</v>
+      </c>
+      <c r="C11" s="16" t="s">
+        <v>99</v>
+      </c>
+      <c r="D11" s="16" t="s">
+        <v>98</v>
+      </c>
+      <c r="E11" s="16" t="s">
+        <v>97</v>
+      </c>
+      <c r="F11" s="14" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" ht="165" x14ac:dyDescent="0.3">
+      <c r="A12" s="12" t="s">
+        <v>39</v>
+      </c>
+      <c r="B12" s="13" t="s">
+        <v>96</v>
+      </c>
+      <c r="C12" s="13" t="s">
+        <v>95</v>
+      </c>
+      <c r="D12" s="13" t="s">
+        <v>94</v>
+      </c>
+      <c r="E12" s="13" t="s">
+        <v>93</v>
+      </c>
+      <c r="F12" s="17" t="s">
+        <v>75</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A2:E2"/>
+    <mergeCell ref="A1:E1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DEE0BE34-8C74-414A-A3E0-80A90A37687F}">
+  <dimension ref="A1:O7"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="13" customWidth="1"/>
+    <col min="2" max="2" width="16" customWidth="1"/>
+    <col min="3" max="4" width="40" customWidth="1"/>
+    <col min="5" max="6" width="12" customWidth="1"/>
+    <col min="7" max="7" width="11" customWidth="1"/>
+    <col min="8" max="8" width="15" customWidth="1"/>
+    <col min="9" max="9" width="34" customWidth="1"/>
+    <col min="10" max="11" width="40" customWidth="1"/>
+    <col min="12" max="12" width="12" customWidth="1"/>
+    <col min="13" max="13" width="17" customWidth="1"/>
+    <col min="14" max="14" width="15" customWidth="1"/>
+    <col min="15" max="15" width="14" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:15" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="19" t="s">
+        <v>135</v>
+      </c>
+      <c r="B1" s="10"/>
+      <c r="C1" s="10"/>
+      <c r="D1" s="10"/>
+      <c r="E1" s="10"/>
+      <c r="F1" s="10"/>
+      <c r="G1" s="10"/>
+      <c r="H1" s="10"/>
+      <c r="I1" s="10"/>
+      <c r="J1" s="10"/>
+      <c r="K1" s="10"/>
+      <c r="L1" s="10"/>
+      <c r="M1" s="10"/>
+      <c r="N1" s="10"/>
+      <c r="O1" s="10"/>
+    </row>
+    <row r="2" spans="1:15" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="18"/>
+      <c r="B2" s="10"/>
+      <c r="C2" s="10"/>
+      <c r="D2" s="10"/>
+      <c r="E2" s="10"/>
+      <c r="F2" s="10"/>
+      <c r="G2" s="10"/>
+      <c r="H2" s="10"/>
+      <c r="I2" s="10"/>
+      <c r="J2" s="10"/>
+      <c r="K2" s="10"/>
+      <c r="L2" s="10"/>
+      <c r="M2" s="10"/>
+      <c r="N2" s="10"/>
+      <c r="O2" s="10"/>
+    </row>
+    <row r="3" spans="1:15" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="7" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B3" s="7" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C3" s="7" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D3" s="7" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E3" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F3" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G3" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H3" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I3" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J3" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K3" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L3" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M3" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N3" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O3" s="7" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="4" spans="1:15" ht="45" x14ac:dyDescent="0.3">
+      <c r="A4" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="P1" t="s">
+      <c r="B4" s="12" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="2" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
+      <c r="C4" s="13" t="s">
         <v>16</v>
       </c>
-      <c r="B2" t="s">
+      <c r="D4" s="13" t="s">
         <v>17</v>
       </c>
-      <c r="C2" t="s">
+      <c r="E4" s="20" t="s">
         <v>18</v>
       </c>
-      <c r="D2" t="s">
+      <c r="F4" s="20" t="s">
         <v>19</v>
       </c>
-      <c r="E2" t="s">
+      <c r="G4" s="12" t="s">
         <v>20</v>
       </c>
-      <c r="F2" t="s">
+      <c r="H4" s="13" t="s">
+        <v>29</v>
+      </c>
+      <c r="I4" s="13" t="s">
+        <v>144</v>
+      </c>
+      <c r="J4" s="13" t="s">
         <v>21</v>
       </c>
-      <c r="G2" t="s">
+      <c r="K4" s="13" t="s">
         <v>22</v>
       </c>
-      <c r="H2" t="s">
+      <c r="L4" s="13" t="s">
+        <v>23</v>
+      </c>
+      <c r="M4" s="22" t="s">
+        <v>138</v>
+      </c>
+      <c r="N4" s="13" t="s">
+        <v>137</v>
+      </c>
+      <c r="O4" s="22" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="5" spans="1:15" ht="30" x14ac:dyDescent="0.3">
+      <c r="A5" s="15" t="s">
+        <v>25</v>
+      </c>
+      <c r="B5" s="15" t="s">
+        <v>27</v>
+      </c>
+      <c r="C5" s="16" t="s">
+        <v>28</v>
+      </c>
+      <c r="D5" s="16" t="s">
+        <v>143</v>
+      </c>
+      <c r="E5" s="20" t="s">
+        <v>18</v>
+      </c>
+      <c r="F5" s="20" t="s">
+        <v>19</v>
+      </c>
+      <c r="G5" s="15" t="s">
+        <v>20</v>
+      </c>
+      <c r="H5" s="16" t="s">
+        <v>29</v>
+      </c>
+      <c r="I5" s="16" t="s">
+        <v>142</v>
+      </c>
+      <c r="J5" s="16" t="s">
+        <v>30</v>
+      </c>
+      <c r="K5" s="16" t="s">
+        <v>31</v>
+      </c>
+      <c r="L5" s="16" t="s">
+        <v>23</v>
+      </c>
+      <c r="M5" s="21" t="s">
+        <v>138</v>
+      </c>
+      <c r="N5" s="16" t="s">
+        <v>137</v>
+      </c>
+      <c r="O5" s="21" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="6" spans="1:15" ht="45" x14ac:dyDescent="0.3">
+      <c r="A6" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="B6" s="12" t="s">
+        <v>33</v>
+      </c>
+      <c r="C6" s="13" t="s">
         <v>34</v>
       </c>
-      <c r="I2" t="s">
+      <c r="D6" s="13" t="s">
+        <v>35</v>
+      </c>
+      <c r="E6" s="20" t="s">
+        <v>18</v>
+      </c>
+      <c r="F6" s="14" t="s">
+        <v>36</v>
+      </c>
+      <c r="G6" s="12" t="s">
+        <v>20</v>
+      </c>
+      <c r="H6" s="13" t="s">
+        <v>29</v>
+      </c>
+      <c r="I6" s="13" t="s">
+        <v>141</v>
+      </c>
+      <c r="J6" s="13" t="s">
+        <v>37</v>
+      </c>
+      <c r="K6" s="13" t="s">
+        <v>38</v>
+      </c>
+      <c r="L6" s="13" t="s">
         <v>23</v>
       </c>
-      <c r="J2" t="s">
+      <c r="M6" s="22" t="s">
+        <v>138</v>
+      </c>
+      <c r="N6" s="13" t="s">
+        <v>137</v>
+      </c>
+      <c r="O6" s="22" t="s">
         <v>24</v>
       </c>
-      <c r="K2" t="s">
-        <v>25</v>
-      </c>
-      <c r="L2" t="s">
-        <v>26</v>
-      </c>
-      <c r="M2" s="1">
-        <v>46149</v>
-      </c>
-      <c r="N2" t="s">
-        <v>27</v>
-      </c>
-      <c r="O2" t="s">
-        <v>28</v>
-      </c>
-      <c r="P2" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="3" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
+    </row>
+    <row r="7" spans="1:15" ht="45" x14ac:dyDescent="0.3">
+      <c r="A7" s="15" t="s">
+        <v>32</v>
+      </c>
+      <c r="B7" s="15" t="s">
+        <v>39</v>
+      </c>
+      <c r="C7" s="16" t="s">
+        <v>43</v>
+      </c>
+      <c r="D7" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="E7" s="17" t="s">
+        <v>40</v>
+      </c>
+      <c r="F7" s="17" t="s">
+        <v>41</v>
+      </c>
+      <c r="G7" s="15" t="s">
+        <v>20</v>
+      </c>
+      <c r="H7" s="16" t="s">
         <v>29</v>
       </c>
-      <c r="B3" t="s">
-        <v>31</v>
-      </c>
-      <c r="C3" t="s">
-        <v>32</v>
-      </c>
-      <c r="D3" t="s">
-        <v>33</v>
-      </c>
-      <c r="E3" t="s">
-        <v>20</v>
-      </c>
-      <c r="F3" t="s">
-        <v>21</v>
-      </c>
-      <c r="G3" t="s">
-        <v>22</v>
-      </c>
-      <c r="H3" t="s">
-        <v>34</v>
-      </c>
-      <c r="I3" t="s">
-        <v>35</v>
-      </c>
-      <c r="J3" t="s">
-        <v>36</v>
-      </c>
-      <c r="K3" t="s">
-        <v>37</v>
-      </c>
-      <c r="L3" t="s">
-        <v>26</v>
-      </c>
-      <c r="M3" s="1">
-        <v>46149</v>
-      </c>
-      <c r="N3" t="s">
-        <v>27</v>
-      </c>
-      <c r="O3" t="s">
-        <v>28</v>
-      </c>
-      <c r="P3" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="4" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
-        <v>30</v>
-      </c>
-      <c r="B4" t="s">
-        <v>39</v>
-      </c>
-      <c r="C4" t="s">
-        <v>40</v>
-      </c>
-      <c r="D4" t="s">
-        <v>41</v>
-      </c>
-      <c r="E4" t="s">
-        <v>20</v>
-      </c>
-      <c r="F4" t="s">
-        <v>42</v>
-      </c>
-      <c r="G4" t="s">
-        <v>22</v>
-      </c>
-      <c r="H4" t="s">
-        <v>34</v>
-      </c>
-      <c r="I4" t="s">
-        <v>43</v>
-      </c>
-      <c r="J4" t="s">
+      <c r="I7" s="16" t="s">
+        <v>140</v>
+      </c>
+      <c r="J7" s="16" t="s">
         <v>44</v>
       </c>
-      <c r="K4" t="s">
-        <v>45</v>
-      </c>
-      <c r="L4" t="s">
-        <v>26</v>
-      </c>
-      <c r="M4" s="1">
-        <v>46149</v>
-      </c>
-      <c r="N4" t="s">
-        <v>27</v>
-      </c>
-      <c r="O4" t="s">
-        <v>28</v>
-      </c>
-      <c r="P4" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="5" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
-        <v>38</v>
-      </c>
-      <c r="B5" t="s">
-        <v>46</v>
-      </c>
-      <c r="C5" t="s">
-        <v>50</v>
-      </c>
-      <c r="D5" t="s">
-        <v>49</v>
-      </c>
-      <c r="E5" t="s">
-        <v>47</v>
-      </c>
-      <c r="F5" t="s">
-        <v>48</v>
-      </c>
-      <c r="G5" t="s">
-        <v>22</v>
-      </c>
-      <c r="H5" t="s">
-        <v>34</v>
-      </c>
-      <c r="I5" t="s">
-        <v>51</v>
-      </c>
-      <c r="J5" t="s">
-        <v>52</v>
-      </c>
-      <c r="K5" t="s">
-        <v>53</v>
-      </c>
-      <c r="L5" t="s">
-        <v>26</v>
-      </c>
-      <c r="M5" s="1">
-        <v>46149</v>
-      </c>
-      <c r="N5" t="s">
-        <v>27</v>
-      </c>
-      <c r="O5" t="s">
-        <v>28</v>
-      </c>
-      <c r="P5" t="s">
-        <v>28</v>
+      <c r="K7" s="16" t="s">
+        <v>139</v>
+      </c>
+      <c r="L7" s="16" t="s">
+        <v>23</v>
+      </c>
+      <c r="M7" s="21" t="s">
+        <v>138</v>
+      </c>
+      <c r="N7" s="16" t="s">
+        <v>137</v>
+      </c>
+      <c r="O7" s="21" t="s">
+        <v>24</v>
       </c>
     </row>
   </sheetData>
-  <phoneticPr fontId="18" type="noConversion"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <mergeCells count="2">
+    <mergeCell ref="A1:O1"/>
+    <mergeCell ref="A2:O2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
+<clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
+  <clbl:label id="{2f70ad68-4eca-4ffe-ad9d-60bfae449e23}" enabled="1" method="Standard" siteId="{b20a8f4d-0d6a-4f2e-83a2-181c968f8882}" contentBits="0" removed="0"/>
+</clbl:labelList>
 </file>
</xml_diff>